<commit_message>
Week6 final: mutual review with 陈雨昂&霍泓锟, PostgreSQL import, paper review, data fixes
</commit_message>
<xml_diff>
--- a/final/301581_黄山谷捷_三表抽取.xlsx
+++ b/final/301581_黄山谷捷_三表抽取.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_认缴流量" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_股权结构存量" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_schema_cross_check" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,6 +454,11 @@
           <t>原文证据</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -472,7 +478,7 @@
         <v>462.8571</v>
       </c>
       <c r="E2" t="n">
-        <v>462.8571</v>
+        <v>10377.2562</v>
       </c>
       <c r="F2" t="n">
         <v>22.42</v>
@@ -480,6 +486,11 @@
       <c r="G2" t="inlineStr">
         <is>
           <t>2021年9月18日，赛格高技术、上汽科技与黄山供销集团、张俊武、周斌及谷捷有限签署《黄山谷捷散热科技有限公司增资协议》，约定谷捷有限增加注册资本514.2857万元，其中赛格高技术认缴462.8571万元、上汽科技认缴51.4286万元，增资价格为22.42元/注册资本，出资方式为货币。</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>auto</t>
         </is>
       </c>
     </row>
@@ -501,7 +512,7 @@
         <v>51.4286</v>
       </c>
       <c r="E3" t="n">
-        <v>51.4286</v>
+        <v>1153.0292</v>
       </c>
       <c r="F3" t="n">
         <v>22.42</v>
@@ -509,6 +520,11 @@
       <c r="G3" t="inlineStr">
         <is>
           <t>2021年9月18日，赛格高技术、上汽科技与黄山供销集团、张俊武、周斌及谷捷有限签署《黄山谷捷散热科技有限公司增资协议》，约定谷捷有限增加注册资本514.2857万元，其中赛格高技术认缴462.8571万元、上汽科技认缴51.4286万元，增资价格为22.42元/注册资本，出资方式为货币。</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>auto</t>
         </is>
       </c>
     </row>
@@ -530,7 +546,7 @@
         <v>90.2256</v>
       </c>
       <c r="E4" t="n">
-        <v>90.2256</v>
+        <v>2124.8129</v>
       </c>
       <c r="F4" t="n">
         <v>23.55</v>
@@ -538,6 +554,11 @@
       <c r="G4" t="inlineStr">
         <is>
           <t>2022年5月24日，谷捷有限与黄山佳捷签署《黄山谷捷散热科技有限公司增资扩股协议》，新增注册资本90.2256万元由黄山佳捷全额认缴，增资价格为23.55元/注册资本，出资方式为货币。</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>auto</t>
         </is>
       </c>
     </row>
@@ -552,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -606,6 +627,11 @@
           <t>原文证据</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -640,6 +666,11 @@
           <t>Markdown表格: 本次发行后 | 股份公司设立, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -674,6 +705,11 @@
           <t>Markdown表格: 本次发行后 | 股份公司设立, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -708,6 +744,11 @@
           <t>Markdown表格: 本次发行后 | 股份公司设立, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -742,6 +783,11 @@
           <t>Markdown表格: 本次发行后 | 股份公司设立, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -776,6 +822,11 @@
           <t>Markdown表格: 本次发行后 | 股份公司设立, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -810,6 +861,11 @@
           <t>Markdown表格: 本次发行后 | 股份公司设立, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -842,6 +898,11 @@
           <t>Markdown表格: 本次发行后 | 股份公司设立, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -876,6 +937,11 @@
           <t>Markdown表格: 本次发行后 | 股份公司设立, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -910,6 +976,11 @@
           <t>Markdown表格: 本次发行后 | 股份公司设立, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -944,6 +1015,11 @@
           <t>Markdown表格: 本次发行后 | 股份公司设立, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -976,6 +1052,11 @@
           <t>Markdown表格: 本次发行后 | 股份公司设立, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1010,6 +1091,11 @@
           <t>Markdown表格: 4、2021 年 11 月，第一次增资，增资至 1,714.2857 万元 | 增资完成后, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1044,6 +1130,11 @@
           <t>Markdown表格: 4、2021 年 11 月，第一次增资，增资至 1,714.2857 万元 | 增资完成后, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1078,6 +1169,11 @@
           <t>Markdown表格: 4、2021 年 11 月，第一次增资，增资至 1,714.2857 万元 | 增资完成后, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1112,6 +1208,11 @@
           <t>Markdown表格: 4、2021 年 11 月，第一次增资，增资至 1,714.2857 万元 | 增资完成后, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1146,6 +1247,11 @@
           <t>Markdown表格: 4、2021 年 11 月，第一次增资，增资至 1,714.2857 万元 | 增资完成后, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1178,6 +1284,11 @@
           <t>Markdown表格: 4、2021 年 11 月，第一次增资，增资至 1,714.2857 万元 | 增资完成后, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1212,6 +1323,11 @@
           <t>Markdown表格: 5、2022 年 5 月，第二次增资，增资至 1,804.5113 万元 | 增资完成后, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1246,6 +1362,11 @@
           <t>Markdown表格: 5、2022 年 5 月，第二次增资，增资至 1,804.5113 万元 | 增资完成后, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1280,6 +1401,11 @@
           <t>Markdown表格: 5、2022 年 5 月，第二次增资，增资至 1,804.5113 万元 | 增资完成后, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1314,6 +1440,11 @@
           <t>Markdown表格: 5、2022 年 5 月，第二次增资，增资至 1,804.5113 万元 | 增资完成后, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1348,6 +1479,11 @@
           <t>Markdown表格: 5、2022 年 5 月，第二次增资，增资至 1,804.5113 万元 | 增资完成后, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1382,6 +1518,11 @@
           <t>Markdown表格: 5、2022 年 5 月，第二次增资，增资至 1,804.5113 万元 | 增资完成后, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1414,6 +1555,11 @@
           <t>Markdown表格: 5、2022 年 5 月，第二次增资，增资至 1,804.5113 万元 | 增资完成后, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1448,6 +1594,11 @@
           <t>Markdown表格: （二）本次发行前的前十名股东情况 | 本次发行后, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1482,6 +1633,11 @@
           <t>Markdown表格: （二）本次发行前的前十名股东情况 | 本次发行后, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1516,6 +1672,11 @@
           <t>Markdown表格: （二）本次发行前的前十名股东情况 | 本次发行后, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1550,6 +1711,11 @@
           <t>Markdown表格: （二）本次发行前的前十名股东情况 | 本次发行后, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1584,6 +1750,11 @@
           <t>Markdown表格: （二）本次发行前的前十名股东情况 | 本次发行后, 比例合计100.0%</t>
         </is>
       </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1616,6 +1787,594 @@
       <c r="J31" t="inlineStr">
         <is>
           <t>Markdown表格: （二）本次发行前的前十名股东情况 | 本次发行后, 比例合计100.0%</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>markdown_table</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>检查类型</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>检查项</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>公司代码</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>校验条目</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>PDF披露值</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>计算值</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>差异</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>差异率</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>是否在容差范围内</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>校验结果</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>原文证据</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>时点</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>schema</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>股权结构存量</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>301581</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>黄山谷捷 三表抽取</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>文件包含3个sheet</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>schema</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>认缴流量</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>301581</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>subscription=3</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>transfer=3</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>cross_check_total</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>持股比例合计</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>301581</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>各时点持股比例合计</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>500.0000</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>待复核</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>30条快照,比例合计500.00</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>全部时点</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>cross_check_shareholder</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>认购价格验算</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>301581</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>赛格高技术 2021-11-11</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>22.42</v>
+      </c>
+      <c r="F5" t="n">
+        <v>22.42</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2021年9月18日，赛格高技术、上汽科技与黄山供销集团、张俊武、周斌及谷捷有限签署《黄山谷捷散热科技有限公司增资协议》，约定谷捷有限增加注册资本514.2857万元，其中赛格高技术认缴462.857</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>金额÷数量=单价</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2021-11-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>cross_check_shareholder</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>认购价格验算</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>301581</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>上汽科技 2021-11-11</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>22.42</v>
+      </c>
+      <c r="F6" t="n">
+        <v>22.42</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2021年9月18日，赛格高技术、上汽科技与黄山供销集团、张俊武、周斌及谷捷有限签署《黄山谷捷散热科技有限公司增资协议》，约定谷捷有限增加注册资本514.2857万元，其中赛格高技术认缴462.857</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>金额÷数量=单价</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2021-11-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>cross_check_shareholder</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>认购价格验算</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>301581</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>黄山佳捷 2022-05-26</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>23.55</v>
+      </c>
+      <c r="F7" t="n">
+        <v>23.55</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2022年5月24日，谷捷有限与黄山佳捷签署《黄山谷捷散热科技有限公司增资扩股协议》，新增注册资本90.2256万元由黄山佳捷全额认缴，增资价格为23.55元/注册资本，出资方式为货币。</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>金额÷数量=单价</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2022-05-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>cross_check_shareholder</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>持股比例合计</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>301581</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>4、2021 年 11 月，第一次增资，增资至 1,714.2857 万元 | 增资完成后 (5名股东)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>100.0000%</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0.0000%</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>合计100.00%</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>4、2021 年 11 月，第一次增资，增资至 1,714.2857 万元 | 增资完成后</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>cross_check_shareholder</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>持股比例合计</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>301581</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>5、2022 年 5 月，第二次增资，增资至 1,804.5113 万元 | 增资完成后 (6名股东)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>100.0000%</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0.0000%</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>合计100.00%</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>5、2022 年 5 月，第二次增资，增资至 1,804.5113 万元 | 增资完成后</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>cross_check_shareholder</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>持股比例合计</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>301581</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>本次发行后 | 股份公司设立 (9名股东)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>200.0000%</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>100.0000%</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>待复核</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>合计200.00%</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>本次发行后 | 股份公司设立</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>cross_check_shareholder</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>持股比例合计</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>301581</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>（二）本次发行前的前十名股东情况 | 本次发行后 (6名股东)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>100.0000%</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>0.0000%</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>合计100.00%</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>（二）本次发行前的前十名股东情况 | 本次发行后</t>
         </is>
       </c>
     </row>

</xml_diff>